<commit_message>
exp: results of 9/24
</commit_message>
<xml_diff>
--- a/MLD01e_Results/Table03_DataSummaryAction_RiskReductionPast25.xlsx
+++ b/MLD01e_Results/Table03_DataSummaryAction_RiskReductionPast25.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5306,37 +5306,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="1" t="inlineStr">
-        <is>
-          <t>Total Money Loss (NRs) due to Drought</t>
-        </is>
-      </c>
-      <c r="B158" t="n">
-        <v>11568</v>
-      </c>
-      <c r="C158" t="n">
-        <v>8568.913468188106</v>
-      </c>
-      <c r="D158" t="n">
-        <v>71176.71615122071</v>
-      </c>
-      <c r="E158" t="n">
-        <v>0</v>
-      </c>
-      <c r="F158" t="n">
-        <v>0</v>
-      </c>
-      <c r="G158" t="n">
-        <v>0</v>
-      </c>
-      <c r="H158" t="n">
-        <v>0</v>
-      </c>
-      <c r="I158" t="n">
-        <v>5000000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>